<commit_message>
Guard the dashboard, the PO archive and the FBR hint lookups
Three routes took a companyId and never checked it. The dashboard's own
comment said it trusted an upstream guard that does not exist, so any signed-in
user could read another company's sales, its clients by name and its stock.
The PO import archive listed and downloaded other tenants' purchase orders by
id. The two HS hint endpoints can spend the named company's FBR token.

Found by building a demo environment and asking for other companies' data as a
freshly created user, which is now a script and a project-local skill.

Also: the shipped opening-stock sample carried a live client's GD numbers,
product names and costs, in a file served publicly. Both sample workbooks are
generated from fictional data now, and Import Costing has a sample of its own.
</commit_message>
<xml_diff>
--- a/myapp-frontend/public/templates/opening-stock-template.xlsx
+++ b/myapp-frontend/public/templates/opening-stock-template.xlsx
@@ -17,8 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0.000"/>
+    <numFmt numFmtId="165" formatCode="0.##%"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -99,7 +100,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -121,6 +122,8 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -486,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG8"/>
+  <dimension ref="A1:AG13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -725,53 +728,53 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>KAPE-HC-64239</t>
+          <t>DEMO-HC-100245</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>13-04-2026</t>
+          <t>12-03-2026</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>8423</t>
+          <t>8482</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>8423.9000</t>
+          <t>8482.1000</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>WEIGHT SCALE PARTS, PLASTIC</t>
+          <t>Industrial Bearing 6204</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>Weight Scale</t>
+          <t>Bearings</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
-        <v>498.777888</v>
+        <v>1250</v>
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>Kg</t>
+          <t>Pcs</t>
         </is>
       </c>
       <c r="J4" s="8" t="n">
-        <v>4037</v>
+        <v>480</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>2013566.33</v>
-      </c>
-      <c r="L4" s="9" t="n">
+        <v>600000</v>
+      </c>
+      <c r="L4" s="17" t="n">
         <v>0.18</v>
       </c>
       <c r="M4" s="7" t="n">
-        <v>362441.94</v>
+        <v>108000</v>
       </c>
       <c r="N4" s="8" t="n">
         <v>0</v>
@@ -779,23 +782,23 @@
       <c r="O4" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="P4" s="9" t="n">
+      <c r="P4" s="17" t="n">
         <v>0.18</v>
       </c>
       <c r="Q4" s="7" t="n">
         <v>0</v>
       </c>
       <c r="R4" s="10" t="n">
-        <v>4037</v>
+        <v>480</v>
       </c>
       <c r="S4" s="11" t="n">
-        <v>2013566.33</v>
-      </c>
-      <c r="T4" s="12" t="n">
+        <v>600000</v>
+      </c>
+      <c r="T4" s="18" t="n">
         <v>0.18</v>
       </c>
       <c r="U4" s="7" t="n">
-        <v>362441.94</v>
+        <v>108000</v>
       </c>
     </row>
     <row r="5">
@@ -806,53 +809,53 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>KAPE-HC-64239</t>
+          <t>DEMO-HC-100245</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>13-04-2026</t>
+          <t>12-03-2026</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>9616</t>
+          <t>8482</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>9616.1000</t>
+          <t>8482.1000</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>PLASTIC ATOMIZER</t>
+          <t>Industrial Bearing 6205</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>Automizer</t>
+          <t>Bearings</t>
         </is>
       </c>
       <c r="H5" s="7" t="n">
-        <v>2438.7608</v>
+        <v>1480</v>
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>Kg</t>
+          <t>Pcs</t>
         </is>
       </c>
       <c r="J5" s="8" t="n">
-        <v>400</v>
+        <v>320</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>975504.3199999999</v>
-      </c>
-      <c r="L5" s="9" t="n">
-        <v>0.25</v>
+        <v>473600</v>
+      </c>
+      <c r="L5" s="17" t="n">
+        <v>0.18</v>
       </c>
       <c r="M5" s="7" t="n">
-        <v>243876.08</v>
+        <v>85248</v>
       </c>
       <c r="N5" s="8" t="n">
         <v>0</v>
@@ -860,23 +863,23 @@
       <c r="O5" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="P5" s="9" t="n">
-        <v>0.25</v>
+      <c r="P5" s="17" t="n">
+        <v>0.18</v>
       </c>
       <c r="Q5" s="7" t="n">
         <v>0</v>
       </c>
       <c r="R5" s="10" t="n">
-        <v>400</v>
+        <v>320</v>
       </c>
       <c r="S5" s="11" t="n">
-        <v>975504.3199999999</v>
-      </c>
-      <c r="T5" s="12" t="n">
-        <v>0.25</v>
+        <v>473600</v>
+      </c>
+      <c r="T5" s="18" t="n">
+        <v>0.18</v>
       </c>
       <c r="U5" s="7" t="n">
-        <v>243876.08</v>
+        <v>85248</v>
       </c>
     </row>
     <row r="6">
@@ -887,102 +890,513 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>KAPW-HC-173918</t>
+          <t>DEMO-HC-100245</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>25-03-2026</t>
+          <t>12-03-2026</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>8482</t>
+          <t>4009</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>8482.9990</t>
+          <t>4009.2200</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>ADAPTER SLEEVE</t>
+          <t>Hydraulic Hose 1/2 inch</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Machines &amp; Electronics</t>
+          <t>Hydraulics</t>
         </is>
       </c>
       <c r="H6" s="7" t="n">
-        <v>765.476723</v>
+        <v>615.5</v>
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
+          <t>Mtr</t>
+        </is>
+      </c>
+      <c r="J6" s="8" t="n">
+        <v>900</v>
+      </c>
+      <c r="K6" s="7" t="n">
+        <v>553950</v>
+      </c>
+      <c r="L6" s="17" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="M6" s="7" t="n">
+        <v>99711</v>
+      </c>
+      <c r="N6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" s="17" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="Q6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" s="10" t="n">
+        <v>900</v>
+      </c>
+      <c r="S6" s="11" t="n">
+        <v>553950</v>
+      </c>
+      <c r="T6" s="18" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="U6" s="7" t="n">
+        <v>99711</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>DEMO-HC-100311</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>04-05-2026</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>7318</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>7318.1510</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Stainless Steel Bolt M10</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Fasteners</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="n">
+        <v>372.25</v>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
           <t>Kg</t>
         </is>
       </c>
-      <c r="J6" s="8" t="n">
-        <v>1253</v>
-      </c>
-      <c r="K6" s="7" t="n">
-        <v>959142.33</v>
-      </c>
-      <c r="L6" s="9" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="M6" s="7" t="n">
-        <v>172645.62</v>
-      </c>
-      <c r="N6" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" s="9" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="Q6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="R6" s="10" t="n">
-        <v>1253</v>
-      </c>
-      <c r="S6" s="11" t="n">
-        <v>959142.33</v>
-      </c>
-      <c r="T6" s="12" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="U6" s="7" t="n">
-        <v>172645.62</v>
+      <c r="J7" s="8" t="n">
+        <v>1250</v>
+      </c>
+      <c r="K7" s="7" t="n">
+        <v>465312.5</v>
+      </c>
+      <c r="L7" s="17" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="M7" s="7" t="n">
+        <v>83756.25</v>
+      </c>
+      <c r="N7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" s="17" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="Q7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" s="10" t="n">
+        <v>1250</v>
+      </c>
+      <c r="S7" s="11" t="n">
+        <v>465312.5</v>
+      </c>
+      <c r="T7" s="18" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="U7" s="7" t="n">
+        <v>83756.25</v>
       </c>
     </row>
     <row r="8">
-      <c r="I8" s="13" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>DEMO-HC-100311</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>04-05-2026</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>8544</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>8544.4990</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>Electrical Cable 2.5mm</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Cables</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="n">
+        <v>148.75</v>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>Mtr</t>
+        </is>
+      </c>
+      <c r="J8" s="8" t="n">
+        <v>4000</v>
+      </c>
+      <c r="K8" s="7" t="n">
+        <v>595000</v>
+      </c>
+      <c r="L8" s="17" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="M8" s="7" t="n">
+        <v>107100</v>
+      </c>
+      <c r="N8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" s="17" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="Q8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" s="10" t="n">
+        <v>4000</v>
+      </c>
+      <c r="S8" s="11" t="n">
+        <v>595000</v>
+      </c>
+      <c r="T8" s="18" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="U8" s="7" t="n">
+        <v>107100</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>DEMO-HC-100311</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>04-05-2026</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>6116</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>6116.1000</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Safety Gloves Coated</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Safety</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="n">
+        <v>265</v>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>Pcs</t>
+        </is>
+      </c>
+      <c r="J9" s="8" t="n">
+        <v>1500</v>
+      </c>
+      <c r="K9" s="7" t="n">
+        <v>397500</v>
+      </c>
+      <c r="L9" s="17" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="M9" s="7" t="n">
+        <v>71550</v>
+      </c>
+      <c r="N9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" s="17" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="Q9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" s="10" t="n">
+        <v>1500</v>
+      </c>
+      <c r="S9" s="11" t="n">
+        <v>397500</v>
+      </c>
+      <c r="T9" s="18" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="U9" s="7" t="n">
+        <v>71550</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>DEMO-HC-100388</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>21-06-2026</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>2710</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>2710.1951</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Machine Oil 20W 5L</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Lubricants</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="n">
+        <v>985</v>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>Ltr</t>
+        </is>
+      </c>
+      <c r="J10" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="K10" s="7" t="n">
+        <v>591000</v>
+      </c>
+      <c r="L10" s="17" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="M10" s="7" t="n">
+        <v>147750</v>
+      </c>
+      <c r="N10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" s="17" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="Q10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" s="10" t="n">
+        <v>600</v>
+      </c>
+      <c r="S10" s="11" t="n">
+        <v>591000</v>
+      </c>
+      <c r="T10" s="18" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="U10" s="7" t="n">
+        <v>147750</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>DEMO-HC-100388</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>21-06-2026</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>4016</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>4016.9390</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Rubber O-Ring Seal 25mm</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Seals</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>42.8</v>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>Pcs</t>
+        </is>
+      </c>
+      <c r="J11" s="8" t="n">
+        <v>2500</v>
+      </c>
+      <c r="K11" s="7" t="n">
+        <v>107000</v>
+      </c>
+      <c r="L11" s="17" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="M11" s="7" t="n">
+        <v>19260</v>
+      </c>
+      <c r="N11" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" s="17" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="Q11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" s="10" t="n">
+        <v>2500</v>
+      </c>
+      <c r="S11" s="11" t="n">
+        <v>107000</v>
+      </c>
+      <c r="T11" s="18" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="U11" s="7" t="n">
+        <v>19260</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="I13" s="13" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="J8" s="14" t="n">
-        <v>5690</v>
-      </c>
-      <c r="K8" s="15" t="n">
-        <v>3948212.98</v>
-      </c>
-      <c r="M8" s="15" t="n">
-        <v>778963.64</v>
-      </c>
-      <c r="R8" s="14" t="n">
-        <v>5690</v>
-      </c>
-      <c r="S8" s="15" t="n">
-        <v>3948212.98</v>
-      </c>
-      <c r="U8" s="15" t="n">
-        <v>778963.64</v>
+      <c r="J13" s="14">
+        <f>SUM(J4:J11)</f>
+        <v/>
+      </c>
+      <c r="K13" s="15">
+        <f>SUM(K4:K11)</f>
+        <v/>
+      </c>
+      <c r="M13" s="15">
+        <f>SUM(M4:M11)</f>
+        <v/>
+      </c>
+      <c r="R13" s="14">
+        <f>SUM(R4:R11)</f>
+        <v/>
+      </c>
+      <c r="S13" s="15">
+        <f>SUM(S4:S11)</f>
+        <v/>
+      </c>
+      <c r="U13" s="15">
+        <f>SUM(U4:U11)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -1017,9 +1431,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="B11" t="inlineStr"/>
-    </row>
+    <row r="11"/>
     <row r="12">
       <c r="B12" t="inlineStr">
         <is>
@@ -1034,9 +1446,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" t="inlineStr"/>
-    </row>
+    <row r="14"/>
     <row r="15">
       <c r="B15" s="16" t="inlineStr">
         <is>
@@ -1072,9 +1482,7 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" t="inlineStr"/>
-    </row>
+    <row r="20"/>
     <row r="21">
       <c r="B21" s="16" t="inlineStr">
         <is>
@@ -1131,9 +1539,7 @@
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="B29" t="inlineStr"/>
-    </row>
+    <row r="29"/>
     <row r="30">
       <c r="B30" s="16" t="inlineStr">
         <is>
@@ -1169,9 +1575,7 @@
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="B35" t="inlineStr"/>
-    </row>
+    <row r="35"/>
     <row r="36">
       <c r="B36" s="16" t="inlineStr">
         <is>

</xml_diff>